<commit_message>
Update manager briefing: add original text and Korean translation columns
Added two columns (원문 내용, 원문 번역) to the left of the issue title
column in the pre-briefing Excel for direct contract clause reference.

https://claude.ai/code/session_0145f7G6Rt9vErLbSt79jyHP
</commit_message>
<xml_diff>
--- a/부장님_사전보고_OEM계약_핵심항목.xlsx
+++ b/부장님_사전보고_OEM계약_핵심항목.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,6 +55,16 @@
       <sz val="8"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <color rgb="001A5276"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <color rgb="00145A32"/>
+      <sz val="8"/>
+    </font>
+    <font>
       <name val="맑은 고딕"/>
       <b val="1"/>
       <color rgb="00000000"/>
@@ -84,7 +94,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -113,7 +123,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FAFCFE"/>
+        <fgColor rgb="00FDECEA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAFAF1"/>
       </patternFill>
     </fill>
     <fill>
@@ -123,12 +138,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDFDFD"/>
+        <fgColor rgb="00E74C3C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E74C3C"/>
+        <fgColor rgb="00FDEDEC"/>
       </patternFill>
     </fill>
     <fill>
@@ -138,17 +153,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDFEFE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FFFDE7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FDEDEC"/>
       </patternFill>
     </fill>
   </fills>
@@ -192,7 +197,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -212,52 +217,76 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -625,18 +654,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:K13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="36" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
+    <col width="32" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -646,14 +677,14 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1">
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>아래 10개 항목은 법무 검토 결과 중 대상웰라이프 측 입장에서 사업 전략·재무·공급 안정성에 중대한 영향을 미치는 사항으로, 협상 전 부장님의 방향성 결정이 필요한 항목입니다.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
+          <t>법무 검토 결과 중 사업 전략·재무·공급 안정성에 중대한 영향을 미치는 10개 항목 – 협상 전 부장님의 방향성 결정이 필요합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>No.</t>
@@ -671,36 +702,46 @@
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
+          <t>원문 내용 (계약서 원문)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>원문 번역</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
           <t>이슈 제목</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>이슈 상세 내용</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>리스크 분석</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>대응 방향</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="J3" s="3" t="inlineStr">
         <is>
           <t>권고 대안 문구</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="K3" s="3" t="inlineStr">
         <is>
           <t>부장님 의사결정 포인트</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="110" customHeight="1">
+    <row r="4" ht="100" customHeight="1">
       <c r="A4" s="4" t="n">
         <v>1</v>
       </c>
@@ -716,42 +757,51 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
+          <t>In case the Client fails to meet the Binding part of the Rolling Forecast specified in Clause 2.2(f), the Client shall pay to the Contract Manufacturer the Conversion Fee for the value of quantity of Products not purchased but should have been purchased by the Client according to the quantities set forth for the Binding 3 months of the Rolling Forecast.</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>의뢰인이 제2.2조(f)에 따른 구속력 있는 롤링 포캐스트 수량을 충족하지 못하는 경우, 의뢰인은 구매하지 않았으나 구매했어야 하는 제품 수량 전체에 대한 전환 수수료를 계약 제조업체에게 지급하여야 한다.</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
           <t>Binding Forecast 미달 시 전환 수수료 전액 지급 의무</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>구속력 있는 롤링 포캐스트(최초 3개월) 수량을 구매하지 않을 경우 미구매 수량 전체에 대한 전환 수수료(Conversion Fee)를 100% 지급해야 함.
-초기 거래 단계에서 정확한 판매 예측이 어려운 상황에서 수량 확약이 현실적으로 가능한지 근본적 문제.</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>구속력 있는 롤링 포캐스트(최초 3개월) 수량을 구매하지 않을 경우 미구매 수량 전체에 대한 Conversion Fee를 100% 지급해야 함.
+초기 거래 단계에서 판매 예측이 불확실한 상황에서 수량 확약이 현실적으로 가능한지 근본 문제.</t>
+        </is>
+      </c>
+      <c r="H4" s="10" t="inlineStr">
         <is>
           <t>• 판매 부진 시 생산 취소 불가 → 제품 미판매 + 수수료 이중 부담
 • 신제품 런칭 초기(수요 불확실 구간)에 집중 적용
-• 연간 최대 노출 규모: MOQ 30톤 × 전환 수수료율(미확정)</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>① 최초 6개월 또는 최초 3 batch: Binding 구간 적용 유예 (Trial 기간 설정)
-② Binding 수량 상한 설정: 직전 실제 구매 수량 기준 ±20% 이내만 구속
-③ 미달 시 다음 PO에 carry-forward 허용 (현금 지급 대신 이연)</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>DenEast 수용 가능성 높은 대안:
-"The Binding Forecast obligation shall not apply during the first six (6) months from the Effective Date (Trial Period). During the Trial Period, the Client's purchase obligations shall be on a best-efforts basis only."</t>
-        </is>
-      </c>
-      <c r="I4" s="9" t="inlineStr">
-        <is>
-          <t>Binding 구간 유예 기간(Trial) 및 미달 시 carry-forward 허용 여부 결정 필요</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="110" customHeight="1">
+• 연간 최대 노출 규모: MOQ 30톤 × Conversion Fee율(미확정)</t>
+        </is>
+      </c>
+      <c r="I4" s="10" t="inlineStr">
+        <is>
+          <t>① 최초 6개월 Trial 기간: Binding 구간 적용 유예
+② Binding 수량 상한: 직전 실구매 수량 ±20% 이내만 구속
+③ 미달 시 다음 PO carry-forward 허용 (현금 지급 대신 이연)</t>
+        </is>
+      </c>
+      <c r="J4" s="10" t="inlineStr">
+        <is>
+          <t>"The Binding Forecast obligation shall not apply during the first six (6) months from the Effective Date (Trial Period). Shortfall quantities may be carried forward to the next rolling period in lieu of cash payment."</t>
+        </is>
+      </c>
+      <c r="K4" s="11" t="inlineStr">
+        <is>
+          <t>Binding 구간 Trial 유예 기간 및 carry-forward 허용 여부 승인</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="100" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>2</v>
       </c>
@@ -760,50 +810,59 @@
           <t>🔴🔴 최우선</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>제3.2조</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
-        <is>
-          <t>Conversion Fee 일방적 인상 + 확정 PO 소급 적용</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>DenEast가 90일 사전 통지만으로 단가(Conversion Fee)를 일방 인상 가능.
-원안: 인상 시 대상웰라이프의 선택지는 '수용' 또는 '30일 통지 해지'뿐.
-법무 수정안에도 이미 수락된 PO, 확정된 Binding Forecast에 인상분 적용 여부 불명확.</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>The Contract Manufacturer, subject to ninety (90) days' advance notice to the Client, may revise the Conversion Fee. If the Client is not satisfied with such revision, the Client has the right to terminate this Agreement, subject to thirty (30) days' advance notice to the Contract Manufacturer.</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>계약 제조업체는 의뢰인에게 90일 전 사전 통지를 조건으로 전환 수수료를 변경할 수 있으며, 의뢰인이 이에 만족하지 않는 경우 30일 전 통지로 본 계약을 해지할 수 있다.</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>Conversion Fee 일방 인상 + 확정 PO 소급 적용</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
+          <t>DenEast가 90일 통지만으로 단가를 일방 인상 가능.
+대상웰라이프의 선택지는 '수용' 또는 '30일 통지 해지'뿐.
+이미 수락된 PO·확정 Binding Forecast에 인상분 소급 적용 여부 불명확.</t>
+        </is>
+      </c>
+      <c r="H5" s="10" t="inlineStr">
         <is>
           <t>• 계약 기간 중 단가 통제 불가 → 손익 구조 붕괴 가능
 • '해지하거나 수용하거나' 구조 – 대체 공급업체 확보 전까지 협상력 없음
-• 이미 확정된 주문에 소급 적용 시 즉각적 손실 발생</t>
-        </is>
-      </c>
-      <c r="G5" s="12" t="inlineStr">
+• 확정 주문 소급 적용 시 즉각적 손실 발생</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
         <is>
           <t>① 인상 협의 의무화: 90일 통지 후 60일 내 상호 합의 필요
-② 소급 적용 금지: 통지 전 수락된 PO 및 Binding Forecast는 기존 단가 유지
-③ 인상 상한 설정: 전년도 대비 연 X% 이내 (인플레이션 연동)</t>
-        </is>
-      </c>
-      <c r="H5" s="12" t="inlineStr">
-        <is>
-          <t>권고 문구:
-"Any revision to the Conversion Fee shall require mutual written agreement. The revised fee shall not apply to any Purchase Orders already accepted or Binding Forecast confirmed prior to the effective date of revision."</t>
-        </is>
-      </c>
-      <c r="I5" s="9" t="inlineStr">
-        <is>
-          <t>단가 인상 협의 의무화 및 소급 적용 금지 조항 삽입 여부 승인 필요</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="110" customHeight="1">
+② 소급 적용 금지: 통지 전 수락 PO·Binding Forecast는 기존 단가 유지
+③ 인상 상한 설정: 전년 대비 연 X% 이내 (인플레이션 연동)</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>"Any revision to the Conversion Fee shall require mutual written agreement. The revised fee shall not apply to any Purchase Orders already accepted or Binding Forecast confirmed prior to the effective date of revision."</t>
+        </is>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>단가 인상 협의 의무화 및 소급 적용 금지 조항 삽입 협상 권한 승인</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="100" customHeight="1">
       <c r="A6" s="4" t="n">
         <v>3</v>
       </c>
@@ -814,418 +873,494 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>제5.3조</t>
+          <t>제5.3(a)조</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
+          <t>The Client shall fulfil its outstanding payment obligations to the Contract Manufacturer for all Products accepted by the Client AND all Products which the Contract Manufacturer manufactured under the respective Purchase Orders and the Product Release Date is notified to the Client prior to the termination date of this Agreement.</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>의뢰인은 (a) 의뢰인이 수락한 제품 및 (b) 계약 제조업체가 해당 구매주문서에 따라 제조하고 계약 종료일 전에 Product Release Date를 통지한 제품 모두에 대해 미지급 대금 지급 의무를 이행해야 한다.</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr">
+        <is>
           <t>계약 해지 시 미완성 제품 포함 대금 전액 지급 의무</t>
         </is>
       </c>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>계약 해지 시, 대상웰라이프가 수령한 제품뿐 아니라 DenEast가 생산 중인 PO에 따른 제품(출고 통지만 하면 됨)에 대해서도 대금 전액 지급 의무 발생.
-공급업체 교체 또는 사업 중단 시 막대한 정산 비용 발생 구조.</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>• 90일 해지 통지 기간 중 DenEast가 생산 극대화 후 대금 청구 가능
-• 해지 의사 표명 = 즉각적 대금 부담 발생 구조
+      <c r="G6" s="10" t="inlineStr">
+        <is>
+          <t>해지 시 대상웰라이프가 수령한 제품뿐 아니라 '출고 통지(Product Release Date 통지)'만 하면 미제조분에도 대금 발생.
+90일 해지 통지 기간 중 DenEast가 생산 극대화 후 청구 가능한 구조.</t>
+        </is>
+      </c>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>• 해지 통지 기간 중 DenEast 생산 극대화 → 대규모 대금 청구
+• 해지 의사 표명 = 즉각적 재무 부담 발생 구조
 • 대체 공급업체 전환 결정을 사실상 가로막는 잠금 효과</t>
         </is>
       </c>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>① 해지 시 미수령 제품 대금 지급 범위 한정:
-   - 해지 통지 전 이미 수락된 PO 중 제조 완료·출고 통지 분만
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>① 지급 범위 한정: 해지 통지 前 이미 수락된 PO 중 제조 완료·출고 통지 분만
 ② 해지 통지 후 신규 생산 착수 금지 조항 삽입
-③ 분쟁 시 에스크로 계좌 활용 조항 추가</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
-        <is>
-          <t>수정 문구 (법무 권고안 기반):
-"Upon termination, Client's payment obligation shall be limited to: (a) Products actually received; and (b) Products fully manufactured AND for which Product Release Date has been notified to Client PRIOR to the termination notice date."</t>
-        </is>
-      </c>
-      <c r="I6" s="9" t="inlineStr">
-        <is>
-          <t>해지 시 대금 지급 범위 한정 조항 협상 권한 및 허용 범위 승인</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="110" customHeight="1">
-      <c r="A7" s="13" t="n">
+③ 분쟁 대비 에스크로 계좌 활용 조항 추가</t>
+        </is>
+      </c>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>"Client's payment obligation shall be limited to: (a) Products actually received; and (b) Products fully manufactured AND for which Product Release Date has been notified to Client PRIOR to the termination notice date."</t>
+        </is>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
+        <is>
+          <t>해지 시 대금 지급 범위 한정 조항 협상 허용 범위 및 에스크로 사용 승인</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="100" customHeight="1">
+      <c r="A7" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>🔴 긴급</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>제2.2(c)조 + 별첨IV</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>The MOQ of Product per Purchase Order shall be 30,000 kg of fluid Product (per one formulation) and shall be reflected in number of units as following: [xxx] units of [TetraPaper Format] packs underfilled [xxx] ml or [xxx] units of [TetraPaper Format] packs underfilled [xxx] ml or a combination of the above two.</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>구매주문당 제품의 최소 주문 수량(MOQ)은 액상 제품 30,000kg(배합 1개당)으로 하며, 단위 수량은 실제 제품 밀도에 따라 조정될 수 있는 [xxx]개의 팩 또는 조합으로 반영된다.</t>
+        </is>
+      </c>
+      <c r="F7" s="15" t="inlineStr">
         <is>
           <t>MOQ 30톤/배합 – 그레듀에이션 스킴·분할 생산 미반영</t>
         </is>
       </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="G7" s="16" t="inlineStr">
         <is>
           <t>계약서 MOQ는 '30톤/배합 1종'으로만 명시.
-Matt Tham과 구두 협의된 내용:
+Matt Tham 구두 협의 내용 (계약서 미반영):
   ① 그레듀에이션 스킴: 20톤, 연 4회 이내 분할 생산
-  ② MOQ 30톤: 다른 배합 2종 동시 생산 가능
-이 내용이 계약서에 반영되지 않은 상태.</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="inlineStr">
-        <is>
-          <t>• 구두 합의가 계약서에 없으면 법적 효력 없음
-• 초기 런칭 시 30톤 확약 → 판매 부진 시 재고 과다 발생
-• 유통기한 제품 특성상 재고 소진 실패 시 전량 폐기 리스크</t>
-        </is>
-      </c>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>① 별첨 IV에 그레듀에이션 스킴 명문화:
-   20톤/회, 연 4회 이내, 2종 배합 동시 가능
-② 본생산 전환 기준 명시: trial 완료 후 30톤 기준 적용
-③ 초기 물량: 'best-efforts' 기준 + MOQ 웨이버 조항</t>
-        </is>
-      </c>
-      <c r="H7" s="12" t="inlineStr">
-        <is>
-          <t>별첨 IV 추가 문구:
-"For the first twelve (12) months (Graduation Period), the MOQ shall be 20 metric tons per formulation, with up to four (4) split production runs permitted annually. Two (2) different formulations may be combined to meet the 30MT MOQ threshold."</t>
-        </is>
-      </c>
-      <c r="I7" s="9" t="inlineStr">
+  ② MOQ 30톤: 다른 배합 2종 동시 생산 가능</t>
+        </is>
+      </c>
+      <c r="H7" s="16" t="inlineStr">
+        <is>
+          <t>• 구두 합의는 법적 효력 없음 → 30톤 단일 확약 강제
+• 초기 런칭 30톤 확약 → 판매 부진 시 재고 과다
+• 유통기한 제품 특성상 재고 소진 실패 시 전량 폐기</t>
+        </is>
+      </c>
+      <c r="I7" s="16" t="inlineStr">
+        <is>
+          <t>① 별첨 IV에 그레듀에이션 스킴 명문화 (20톤/회, 연 4회, 2종 배합)
+② 시범 기간 완료 후 30톤 기준 적용으로 전환
+③ 초기 물량 best-efforts 기준 + MOQ 웨이버 조항</t>
+        </is>
+      </c>
+      <c r="J7" s="16" t="inlineStr">
+        <is>
+          <t>"For the first 12 months (Graduation Period), MOQ shall be 20MT per formulation with up to four (4) split production runs annually. Two different formulations may be combined to meet the 30MT threshold."</t>
+        </is>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>Matt Tham 협의 내용의 계약서 반영 범위 및 최종 MOQ 조건 승인</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="110" customHeight="1">
-      <c r="A8" s="13" t="n">
+    <row r="8" ht="100" customHeight="1">
+      <c r="A8" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>🔴 긴급</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>제2.4(d)조</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
+          <t>Both Parties agree that the Client is responsible to make a sufficient prepayment in order to enable the Contract Manufacturer to start procurement of the Materials in the amount that will be additionally stipulated by the Contract Manufacturer in writing.</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>양 당사자는 계약 제조업체가 자재 조달을 시작할 수 있도록 의뢰인이 충분한 선급금을 지급할 책임이 있다는 데 동의한다. 해당 금액은 계약 제조업체가 서면으로 추가 명시하는 금액으로 한다.</t>
+        </is>
+      </c>
+      <c r="F8" s="15" t="inlineStr">
+        <is>
           <t>선급금 기준·상한 없음 – DenEast 일방 통지로 지급 의무 발생</t>
         </is>
       </c>
-      <c r="E8" s="8" t="inlineStr">
-        <is>
-          <t>원자재 조달 착수를 위해 대상웰라이프가 '충분한' 선급금을 지급해야 하나, 금액은 DenEast가 서면으로 통지하는 금액으로 정해짐.
-승인 프로세스, 증빙 제출 의무, 미사용분 반환 의무 모두 불명확.</t>
-        </is>
-      </c>
-      <c r="F8" s="8" t="inlineStr">
-        <is>
-          <t>• DenEast가 과대 선급금 요청 가능 → 운전자본 부담
+      <c r="G8" s="16" t="inlineStr">
+        <is>
+          <t>원자재 조달 착수를 위해 '충분한' 선급금을 지급해야 하나, 금액은 DenEast가 서면 통지하는 금액으로 정해짐.
+승인 프로세스·증빙 제출 의무·미사용분 반환 의무 모두 불명확.</t>
+        </is>
+      </c>
+      <c r="H8" s="16" t="inlineStr">
+        <is>
+          <t>• DenEast 과대 선급금 요청 → 운전자본 부담
 • 미사용 선급금 미반환 시 손실 발생
-• Procurement Plan 없이 착수 → 과도한 원료 조달 후 보관료 추가 발생</t>
-        </is>
-      </c>
-      <c r="G8" s="8" t="inlineStr">
+• Procurement Plan 없이 착수 → 과도 원료 조달 + 보관료 추가</t>
+        </is>
+      </c>
+      <c r="I8" s="16" t="inlineStr">
         <is>
           <t>① Procurement Plan 기준 선급금 산정 의무화
-② 견적서/인보이스 등 증빙 제출 후 Client 서면 승인 조건
+② 견적서·인보이스 증빙 제출 후 Client 서면 승인 조건
 ③ 미사용 잔액 자동 반환 또는 차기 인보이스 상계
-④ 지급 기한: 3일 → 5~10 영업일로 조정</t>
-        </is>
-      </c>
-      <c r="H8" s="8" t="inlineStr">
-        <is>
-          <t>수정 문구 (대응방안 기반):
-"Prepayment shall be based on the mutually approved Procurement Plan with supporting invoices. Any unused balance shall be refunded or set off against the next invoice at Client's option. Payment due within 7 business days of Client's written approval."</t>
-        </is>
-      </c>
-      <c r="I8" s="9" t="inlineStr">
-        <is>
-          <t>선급금 승인 프로세스 내부 확립 및 지급 기한 협상 범위 결정</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="110" customHeight="1">
-      <c r="A9" s="13" t="n">
+④ 지급 기한 3일 → 5~10 영업일로 조정</t>
+        </is>
+      </c>
+      <c r="J8" s="16" t="inlineStr">
+        <is>
+          <t>"Prepayment shall be based on the mutually approved Procurement Plan with supporting invoices/quotes. Unused balance shall be refunded or set off against next invoice. Payment due within 7 business days of Client's written approval."</t>
+        </is>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>선급금 승인 프로세스 확립 및 지급 기한 협상 범위 결정</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="100" customHeight="1">
+      <c r="A9" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>🔴 긴급</t>
         </is>
       </c>
-      <c r="C9" s="10" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>제3.5조</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>The Client shall, within ten (10) days upon receipt of relevant invoice and copy of certificate of insurance (if applicable), reimburse to the Contract Manufacturer the cost of insurance in which the Client is named as additional insured, and which cover all operations and the Products (product liability) within the scope of this Agreement.</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>의뢰인은 관련 송장 및 보험증권 사본 수령 후 10일 이내에 의뢰인이 추가 피보험자(additional insured)로 명시된 보험 비용을 계약 제조업체에게 상환하여야 한다. (제품 운영·제조물 책임 포함)</t>
+        </is>
+      </c>
+      <c r="F9" s="15" t="inlineStr">
         <is>
           <t>제조물 책임 보험 – 전체 보험료 상환 의무 (OEM 발주사 책임)</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>DenEast가 Client를 additional insured로 포함한 보험에 가입하면, 대상웰라이프가 10일 이내에 보험료 전액을 상환해야 함.
-OEM 구조상 제조물 책임은 브랜드사(대상웰라이프) 부담이 크며, 보험 범위·금액 사전 승인 없이 청구 가능.</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>• 보험료 규모 미사전 합의 → 예산 외 비용 발생
+      <c r="G9" s="16" t="inlineStr">
+        <is>
+          <t>DenEast가 Client를 additional insured로 포함한 보험에 가입하면 대상웰라이프가 10일 이내에 보험료 전액을 상환해야 함.
+OEM 구조상 브랜드사(대상웰라이프)의 제조물 책임이 크며, 보험 범위·금액 사전 승인 없이 청구 가능.</t>
+        </is>
+      </c>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>• 보험료 규모 사전 미합의 → 예산 외 비용 발생
 • 제조물 책임 사고 시 1차 보상 주체는 대상웰라이프
 • 보험 범위 불충분 시 추가 손해배상 노출</t>
         </is>
       </c>
-      <c r="G9" s="12" t="inlineStr">
+      <c r="I9" s="16" t="inlineStr">
         <is>
           <t>① 상환 범위: additional insured 추가로 인한 증분 비용만
-② DenEast 일반 운영보험·공장보험은 DenEast 부담
+② DenEast 일반 운영·공장 보험은 DenEast 부담
 ③ 보험 가입 전 Client 사전 서면 승인 의무화
-④ 별도 제조물 책임 보험 가입 검토 (내부)</t>
-        </is>
-      </c>
-      <c r="H9" s="12" t="inlineStr">
-        <is>
-          <t>수정 문구:
-"Client shall reimburse only the reasonable incremental cost of naming Client as additional insured, subject to Client's prior written approval. Contract Manufacturer shall bear all costs of its own general, operational, and facility insurance."</t>
-        </is>
-      </c>
-      <c r="I9" s="9" t="inlineStr">
+④ 별도 제조물 책임 보험 가입 내부 검토</t>
+        </is>
+      </c>
+      <c r="J9" s="16" t="inlineStr">
+        <is>
+          <t>"Client shall reimburse only the reasonable incremental cost of naming Client as additional insured, subject to Client's prior written approval. CM shall bear all costs of its own general, operational, and facility insurance."</t>
+        </is>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
         <is>
           <t>사내 별도 제조물 책임 보험 가입 여부 및 예산 편성 승인</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="110" customHeight="1">
-      <c r="A10" s="13" t="n">
+    <row r="10" ht="100" customHeight="1">
+      <c r="A10" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>🔴 긴급</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>제2.6(a)·(d)조</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>EXW 인도 조건 – 베트남 현지 픽업 시점부터 전 리스크 Client 부담</t>
+          <t>Delivery terms shall be Ex-Works (Incoterms 2010) 7 VSIP II-A Street 31, Vietnam Singapore Industrial Park II-A, Vinh Tan Ward, Ho Chi Minh City, Vietnam if otherwise is not agreed by the Parties. Title to the Product(s) will transfer from the Contract Manufacturer to the Client at the time risk of loss transfers pursuant to the delivery terms.</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>인도 조건은 Ex-Works(DenEast 창고)로, 창고 출고 시점부터 소유권·손실 위험 모두 대상웰라이프 이전.
-베트남 현지 포워더 지정, 통관, 운송 전 과정을 직접 관리해야 함.</t>
-        </is>
-      </c>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>• 픽업 전 창고 화재·홍수·도난 등 손실 → Client 부담
-• 8일 초과 보관 시 $1.10/팔레트/일 보관료 자동 발생
+          <t>당사자들이 달리 합의하지 않는 한, 인도 조건은 Incoterms 2010 Ex-Works 조건으로 하며 인도 장소는 베트남 호치민시 DenEast 창고로 한다. 제품에 대한 소유권은 Ex-Works 조건에 따라 손실 위험이 이전되는 시점에 계약 제조업체로부터 의뢰인에게 이전된다.</t>
+        </is>
+      </c>
+      <c r="F10" s="15" t="inlineStr">
+        <is>
+          <t>EXW 인도 조건 – 창고 출고 즉시 전 리스크·소유권 Client 이전</t>
+        </is>
+      </c>
+      <c r="G10" s="16" t="inlineStr">
+        <is>
+          <t>인도 조건 Ex-Works로, 창고 출고 시점부터 소유권·손실 위험 모두 대상웰라이프 이전.
+베트남 현지 포워더 지정·통관·운송 전 과정을 직접 관리해야 함.
+8일 초과 보관 시 $1.10/팔레트/일 보관료 자동 발생.</t>
+        </is>
+      </c>
+      <c r="H10" s="16" t="inlineStr">
+        <is>
+          <t>• 픽업 전 창고 화재·홍수·도난 등 손실 → Client 전액 부담
+• 8일 초과 보관 시 보관료 누적 발생
 • 베트남 현지 물류 인프라 미구축 시 운영 차질</t>
         </is>
       </c>
-      <c r="G10" s="8" t="inlineStr">
+      <c r="I10" s="16" t="inlineStr">
         <is>
           <t>① SCM팀: 베트남 현지 포워더 사전 계약 체결
-② 출고 통지 수령 후 즉각 픽업 일정 확보 체계 구축
-③ 픽업 전 구간 DenEast 창고 보험 가입 확인
+② 출고 통지 즉각 픽업 일정 확보 체계 구축
+③ 픽업 전 구간 창고 보험 가입 확인
 ④ 가능 시 FOB 호치민항으로 인도 조건 변경 협의</t>
         </is>
       </c>
-      <c r="H10" s="8" t="inlineStr">
+      <c r="J10" s="16" t="inlineStr">
         <is>
           <t>협상 우선순위:
 1안(최선): FOB Ho Chi Minh Port
-2안(차선): EXW 유지 + 픽업 전 구간 DenEast 보관 책임·보험 유지 조항
-3안(수용): EXW 유지 + 보관료 면제 기간 연장(8일→14일)</t>
-        </is>
-      </c>
-      <c r="I10" s="9" t="inlineStr">
-        <is>
-          <t>인도 조건(EXW vs FOB) 협상 방향 및 현지 물류 체계 구축 일정 승인</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="110" customHeight="1">
-      <c r="A11" s="15" t="n">
+2안(차선): EXW + 픽업 전 구간 DenEast 보관 책임·보험 유지
+3안(수용): EXW + 보관료 면제 기간 연장(8일→14일)</t>
+        </is>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>인도 조건(EXW→FOB) 협상 방향 및 현지 물류 체계 구축 일정 승인</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="100" customHeight="1">
+      <c r="A11" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="18" t="inlineStr">
         <is>
           <t>🟠 중요</t>
         </is>
       </c>
-      <c r="C11" s="10" t="inlineStr">
+      <c r="C11" s="19" t="inlineStr">
         <is>
           <t>제3.1·3.2조 + 별첨III</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>가격 구조 전반 미확정 – Conversion Fee·부대수수료·VAT 공란</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>① Conversion Fee: 그레듀에이션(시범) vs 본생산 단가 상이하나 별첨 미기재
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>The Purchase Price shall be composed of the following components (all amounts in USD excluding VAT. The VAT under the laws of Vietnam is [ ] percent ([ ]%). ): i. Conversion Fee  ii. Packaging Material cost  iii. Standard Material Price  iv. Auxiliary Fee (if any)</t>
+        </is>
+      </c>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>구매가격은 다음 구성요소로 구성되며 모든 금액은 USD 기준이고 VAT를 제외한다. 베트남 법률상 VAT율은 공란에 기재한다. 구성: i.전환 수수료  ii.포장재 비용  iii.표준 자재 가격  iv.부대 수수료(해당 시)</t>
+        </is>
+      </c>
+      <c r="F11" s="20" t="inlineStr">
+        <is>
+          <t>가격 구조 전반 미확정 – 단가·부대수수료·VAT 공란</t>
+        </is>
+      </c>
+      <c r="G11" s="21" t="inlineStr">
+        <is>
+          <t>① Conversion Fee: 그레듀에이션 vs 본생산 단가 상이하나 별첨 미기재
 ② Auxiliary Fee: 추가 부대비용 항목·상한 미정
-③ VAT: 베트남 내수 유통 시 VAT 발생 여부·세율 공란
+③ VAT: 베트남 내수 유통 시 발생 여부·세율 공란
 ④ True-up: 실제 원가 vs Standard Material Price 정산 기준 불명확</t>
         </is>
       </c>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t>• 가격 구조 미확정 상태 서명 시 계약 효력은 발생하나 단가 분쟁 예약
-• VAT 미반영 시 실제 구매단가 &gt; 협의 단가 (예: VAT 10% 추가 시)
+      <c r="H11" s="21" t="inlineStr">
+        <is>
+          <t>• 가격 미확정 상태 서명 시 계약 효력 발생 → 단가 분쟁 예약
+• VAT 미반영 시 실제 구매단가 &gt; 협의 단가
 • Auxiliary Fee 무제한 청구 가능 구조</t>
         </is>
       </c>
-      <c r="G11" s="12" t="inlineStr">
-        <is>
-          <t>① 별첨 III 완성 전 서명 금지 (내부 원칙 설정)
+      <c r="I11" s="21" t="inlineStr">
+        <is>
+          <t>① 별첨 III 완성 전 서명 금지 (강제 원칙)
 ② Auxiliary Fee: 항목 열거 + 건당 Client 사전 서면 승인 필수
 ③ VAT: 관세사·세무팀 확인 후 세율 기재
-④ True-up: Procurement Plan 기준 + 증빙 제출 의무화</t>
-        </is>
-      </c>
-      <c r="H11" s="12" t="inlineStr">
-        <is>
-          <t>별첨 III 기재 원칙:
+④ True-up: Procurement Plan 기준 + 증빙 의무화</t>
+        </is>
+      </c>
+      <c r="J11" s="21" t="inlineStr">
+        <is>
+          <t>별첨 III 원칙:
 - Conversion Fee: 시범(20톤) / 본생산(30톤) 구분 단가
-- Auxiliary Fee: 승인된 항목만 청구 가능, 상한 설정
-- VAT: 수출 거래(0%) 또는 내수(10%) 명확히 구분</t>
-        </is>
-      </c>
-      <c r="I11" s="9" t="inlineStr">
-        <is>
-          <t>별첨 III 가격 조건 확정 전 서명 금지 원칙 수립 + 재무/세무팀 검토 지시</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="110" customHeight="1">
-      <c r="A12" s="15" t="n">
+- Auxiliary Fee: 승인된 항목만, 상한 설정
+- VAT: 수출(0%) or 내수(10%) 명확히 구분 기재</t>
+        </is>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>별첨 III 완성 전 서명 금지 원칙 수립 + 재무·세무팀 검토 지시</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="100" customHeight="1">
+      <c r="A12" s="17" t="n">
         <v>9</v>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="18" t="inlineStr">
         <is>
           <t>🟠 중요</t>
         </is>
       </c>
-      <c r="C12" s="6" t="inlineStr">
+      <c r="C12" s="19" t="inlineStr">
         <is>
           <t>제5.1·5.2조</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
+          <t>5.1. Unless earlier terminated, this Agreement shall be effective from the Effective Date and remain in full force and effect for a period of twelve (12) months. This Agreement may only be renewed by explicit mutual written agreement of the Parties.
+5.2. Either Party may terminate this Agreement at any time, without cause, by giving the other Party ninety (90) days' prior written notice.</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>5.1. 본 계약은 조기 해지되지 않는 한 효력 발생일로부터 12개월 동안 유효하며, 당사자들의 명시적인 상호 서면 합의에 의해서만 갱신될 수 있다.
+5.2. 어느 당사자든지 상대방에게 90일 전 사전 서면 통지를 함으로써 사유 없이 본 계약을 해지할 수 있다.</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
           <t>계약 기간 12개월 + 무사유 90일 해지 – 공급 안정성 위협</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr">
-        <is>
-          <t>계약 기간은 12개월, 자동 갱신 없음(명시적 서면 합의 필요).
-양 당사자 모두 90일 사전 통지로 무사유 해지 가능.
-단, 법무 검토: 대체 공급업체 확보 관점에서 일방 해지권은 유리할 수도 있음.</t>
-        </is>
-      </c>
-      <c r="F12" s="8" t="inlineStr">
-        <is>
-          <t>• DenEast 무사유 해지 시 90일 내 대체 공급업체 확보 불가능
-• 제품 단종·단기 공급 중단 → 고객사 클레임
-• 기술이전·BOM 공유 후 해지 시 IP 반환·삭제 담보 불명확</t>
-        </is>
-      </c>
-      <c r="G12" s="8" t="inlineStr">
+      <c r="G12" s="21" t="inlineStr">
+        <is>
+          <t>계약 기간 12개월, 자동 갱신 없음(명시적 서면 합의 필요).
+양 당사자 모두 90일 통지로 무사유 해지 가능.
+법무 검토: 대체 공급업체 확보 관점에서 일방 해지권은 유리할 수도 있음.</t>
+        </is>
+      </c>
+      <c r="H12" s="21" t="inlineStr">
+        <is>
+          <t>• DenEast 무사유 해지 시 90일 내 대체 공급업체 확보 불가
+• 기술이전·BOM 공유 후 해지 시 IP 반환·삭제 담보 불명확
+• 제품 단종·단기 공급 중단 → 고객사 클레임</t>
+        </is>
+      </c>
+      <c r="I12" s="21" t="inlineStr">
         <is>
           <t>① 최소 계약 기간 연장: 12개월 → 24~36개월
-② DenEast의 무사유 해지 제한: 계약 2년 경과 후부터만 허용
+② DenEast 무사유 해지 제한: 계약 2년 경과 후부터만 허용
 ③ 해지 통지 기간 연장: 90일 → 180일
-④ 해지 시 기술자료·BOM 반환 및 삭제 확인서 수령 조항 추가</t>
-        </is>
-      </c>
-      <c r="H12" s="8" t="inlineStr">
-        <is>
-          <t>협상 대안:
-"Notwithstanding Clause 5.2, the Contract Manufacturer may not terminate for convenience during the first 24 months. Thereafter, termination notice period shall be 180 days. Upon termination, CM shall return/destroy all Client's Confidential Information and confirm in writing."</t>
-        </is>
-      </c>
-      <c r="I12" s="9" t="inlineStr">
+④ 해지 시 기술자료·BOM 반환·삭제 확인서 조항 추가</t>
+        </is>
+      </c>
+      <c r="J12" s="21" t="inlineStr">
+        <is>
+          <t>"CM may not terminate for convenience during the first 24 months. Thereafter, termination notice period shall be 180 days. Upon termination, CM shall return/destroy all Client's Confidential Information and provide written confirmation."</t>
+        </is>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>최소 계약 기간(2~3년) 및 해지 통지 기간(180일) 협상 방향 승인</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="110" customHeight="1">
-      <c r="A13" s="15" t="n">
+    <row r="13" ht="100" customHeight="1">
+      <c r="A13" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="18" t="inlineStr">
         <is>
           <t>🟠 중요</t>
         </is>
       </c>
-      <c r="C13" s="10" t="inlineStr">
-        <is>
-          <t>별첨I + 기술이전 조항</t>
-        </is>
-      </c>
-      <c r="D13" s="11" t="inlineStr">
-        <is>
-          <t>Appendix I(제품사양·BOM·제조공정) 미완성 – 서명 전 완료 필수</t>
-        </is>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>OEM 계약의 핵심인 별첨 I(제품 사양, BOM, 배합 지시서, 생산 공정도)이 현재 공란 상태.
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>별첨 I + 기술이전 조항</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>APPENDIX I – The Contract Manufacturer shall manufacture the Product(s) in accordance with the applicable Bill of Materials, Production Flowchart and Mixing Instruction as specified in Appendix I of this Agreement and approved by the Client during the technical transfer process. [현재 전체 공란]</t>
+        </is>
+      </c>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>별첨 I – 계약 제조업체는 본 계약서 Appendix I에 명시되고 기술이전 과정에서 Client가 승인한 BOM, 생산 공정도 및 배합 지시서에 따라 제품을 제조해야 한다. [현재 전체 공란 상태]</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>Appendix I (제품사양·BOM·제조공정) 미완성 – 서명 전 필수 완료</t>
+        </is>
+      </c>
+      <c r="G13" s="21" t="inlineStr">
+        <is>
+          <t>OEM 계약의 핵심인 별첨 I(제품 사양, BOM, 배합 지시서, 생산 공정도)이 현재 공란.
 별첨 I 없이 계약 효력 발생 시:
   - 품질 기준 분쟁 시 판단 근거 없음
-  - DenEast가 사양 일방 해석 가능</t>
-        </is>
-      </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>• 품질 불량 발생 시 책임 소재 불명 → Client 책임으로 전가 가능
-• BOM 미확정 → Standard Material Price, 선급금 산정 기준 없음
+  - DenEast가 사양 일방 해석 가능
+  - 가격 구조(Standard Material Price, 선급금) 산정 기준도 없음</t>
+        </is>
+      </c>
+      <c r="H13" s="21" t="inlineStr">
+        <is>
+          <t>• 품질 불량 시 책임 소재 불명 → Client 책임 전가 가능
+• BOM 미확정 → 단가·선급금 산정 기준 없음
 • 기술이전 내용 미기재 → IP 보호 불완전</t>
         </is>
       </c>
-      <c r="G13" s="12" t="inlineStr">
-        <is>
-          <t>① 서명 조건: 별첨 I 완성 후에만 서명 진행 (강제 조건)
+      <c r="I13" s="21" t="inlineStr">
+        <is>
+          <t>① 서명 조건: 별첨 I 완성 후에만 서명 진행 (강제 원칙)
 ② BOM 수령 후 원가 재검토 (재무팀)
 ③ 기술이전 범위·절차 별첨에 명시
 ④ 별첨 I 변경 시 양방 서면 합의 필요 조항 확인</t>
         </is>
       </c>
-      <c r="H13" s="12" t="inlineStr">
-        <is>
-          <t>단기 대안(부득이 서명 시):
-"Appendix I shall be completed and mutually executed within 30 days of Effective Date as a condition to production commencement. Production shall not commence until Appendix I is fully executed."</t>
-        </is>
-      </c>
-      <c r="I13" s="9" t="inlineStr">
+      <c r="J13" s="21" t="inlineStr">
+        <is>
+          <t>부득이 서명 시:
+"Appendix I shall be completed and mutually executed within 30 days of the Effective Date as a condition to production commencement. No production shall commence until Appendix I is fully executed by both Parties."</t>
+        </is>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
         <is>
           <t>별첨 I 완성 전 서명 금지 원칙 확립 + BOM 수령 일정 확인</t>
         </is>
@@ -1233,8 +1368,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1246,256 +1381,311 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>부장님 의사결정 체크리스트 – 협상 전 확인 필요 사항</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="18" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="B2" s="18" t="inlineStr">
-        <is>
-          <t>이슈</t>
-        </is>
-      </c>
-      <c r="C2" s="18" t="inlineStr">
+      <c r="B2" s="23" t="inlineStr">
+        <is>
+          <t>우선순위</t>
+        </is>
+      </c>
+      <c r="C2" s="23" t="inlineStr">
+        <is>
+          <t>이슈 제목</t>
+        </is>
+      </c>
+      <c r="D2" s="23" t="inlineStr">
         <is>
           <t>필요한 결정 내용</t>
         </is>
       </c>
-      <c r="D2" s="18" t="inlineStr">
-        <is>
-          <t>결정 방향
-(기재)</t>
-        </is>
-      </c>
-      <c r="E2" s="18" t="inlineStr">
+      <c r="E2" s="23" t="inlineStr">
+        <is>
+          <t>결정 방향 (기재)</t>
+        </is>
+      </c>
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>기한</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1">
+    <row r="3" ht="28" customHeight="1">
       <c r="A3" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="19" t="inlineStr">
-        <is>
-          <t>Binding Forecast 구속 완화</t>
-        </is>
-      </c>
-      <c r="C3" s="20" t="inlineStr">
-        <is>
-          <t>Trial 기간(6개월) 유예 및 미달 시 carry-forward 허용 여부</t>
-        </is>
-      </c>
-      <c r="D3" s="21" t="inlineStr"/>
-      <c r="E3" s="22" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>🔴🔴 최우선</t>
+        </is>
+      </c>
+      <c r="C3" s="25" t="inlineStr">
+        <is>
+          <t>Binding Forecast 미달 전환 수수료</t>
+        </is>
+      </c>
+      <c r="D3" s="26" t="inlineStr">
+        <is>
+          <t>Trial 6개월 유예 및 carry-forward 허용 여부</t>
+        </is>
+      </c>
+      <c r="E3" s="27" t="inlineStr"/>
+      <c r="F3" s="28" t="inlineStr">
         <is>
           <t>서명 전</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1">
+    <row r="4" ht="28" customHeight="1">
       <c r="A4" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="19" t="inlineStr">
-        <is>
-          <t>Conversion Fee 단가 보호</t>
-        </is>
-      </c>
-      <c r="C4" s="20" t="inlineStr">
-        <is>
-          <t>단가 인상 협의 의무화 + 확정 PO 소급 적용 금지 협상 권한</t>
-        </is>
-      </c>
-      <c r="D4" s="21" t="inlineStr"/>
-      <c r="E4" s="22" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>🔴🔴 최우선</t>
+        </is>
+      </c>
+      <c r="C4" s="25" t="inlineStr">
+        <is>
+          <t>Conversion Fee 일방 인상</t>
+        </is>
+      </c>
+      <c r="D4" s="26" t="inlineStr">
+        <is>
+          <t>협의 의무화 + 확정 PO 소급 금지 협상 권한</t>
+        </is>
+      </c>
+      <c r="E4" s="27" t="inlineStr"/>
+      <c r="F4" s="28" t="inlineStr">
         <is>
           <t>서명 전</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
+    <row r="5" ht="28" customHeight="1">
       <c r="A5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>🔴🔴 최우선</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>해지 시 대금 지급 범위</t>
         </is>
       </c>
-      <c r="C5" s="20" t="inlineStr">
-        <is>
-          <t>출고 통지 완료분만 지급 한정 조항 협상 허용 범위</t>
-        </is>
-      </c>
-      <c r="D5" s="21" t="inlineStr"/>
-      <c r="E5" s="22" t="inlineStr">
+      <c r="D5" s="26" t="inlineStr">
+        <is>
+          <t>출고 통지 완료분만 지급 한정 협상 허용 범위</t>
+        </is>
+      </c>
+      <c r="E5" s="27" t="inlineStr"/>
+      <c r="F5" s="28" t="inlineStr">
         <is>
           <t>서명 전</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="13" t="n">
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>MOQ / 그레듀에이션 스킴</t>
-        </is>
-      </c>
-      <c r="C6" s="20" t="inlineStr">
-        <is>
-          <t>20톤 시범 + 30톤 본생산 구분, 2종 배합 허용 명문화 승인</t>
-        </is>
-      </c>
-      <c r="D6" s="21" t="inlineStr"/>
-      <c r="E6" s="22" t="inlineStr">
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>🔴 긴급</t>
+        </is>
+      </c>
+      <c r="C6" s="25" t="inlineStr">
+        <is>
+          <t>MOQ 그레듀에이션 스킴</t>
+        </is>
+      </c>
+      <c r="D6" s="26" t="inlineStr">
+        <is>
+          <t>20톤 시범+30톤 본생산 구분, 2종 배합 허용 명문화</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr"/>
+      <c r="F6" s="28" t="inlineStr">
         <is>
           <t>서명 전</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="13" t="n">
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="12" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>🔴 긴급</t>
+        </is>
+      </c>
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>선급금 프로세스</t>
         </is>
       </c>
-      <c r="C7" s="20" t="inlineStr">
-        <is>
-          <t>Procurement Plan 기준 + 5~10 영업일 지급 기한 협상 승인</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr"/>
-      <c r="E7" s="22" t="inlineStr">
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>Procurement Plan 기준 + 5~10 영업일 지급 기한</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr"/>
+      <c r="F7" s="28" t="inlineStr">
         <is>
           <t>서명 전</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="13" t="n">
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="19" t="inlineStr">
+      <c r="B8" s="29" t="inlineStr">
+        <is>
+          <t>🔴 긴급</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
         <is>
           <t>제조물 책임 보험</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
-        <is>
-          <t>증분 비용만 상환 협상 + 사내 별도 보험 가입 예산 승인</t>
-        </is>
-      </c>
-      <c r="D8" s="21" t="inlineStr"/>
-      <c r="E8" s="22" t="inlineStr">
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>증분 비용만 상환 + 사내 별도 보험 예산 승인</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr"/>
+      <c r="F8" s="28" t="inlineStr">
         <is>
           <t>서명 전</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="13" t="n">
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="19" t="inlineStr">
-        <is>
-          <t>인도 조건 (EXW→FOB)</t>
-        </is>
-      </c>
-      <c r="C9" s="20" t="inlineStr">
-        <is>
-          <t>FOB 호치민 또는 EXW 보관 기간 연장(14일) 협상 방향 승인</t>
-        </is>
-      </c>
-      <c r="D9" s="21" t="inlineStr"/>
-      <c r="E9" s="22" t="inlineStr">
+      <c r="B9" s="29" t="inlineStr">
+        <is>
+          <t>🔴 긴급</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>EXW 인도 조건</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>FOB 협상 또는 EXW 보관 기간 연장 방향</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr"/>
+      <c r="F9" s="28" t="inlineStr">
         <is>
           <t>서명 전</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="15" t="n">
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>가격 구조 완성</t>
-        </is>
-      </c>
-      <c r="C10" s="20" t="inlineStr">
-        <is>
-          <t>별첨 III 완성 전 서명 금지 원칙 + 재무/세무팀 검토 지시</t>
-        </is>
-      </c>
-      <c r="D10" s="21" t="inlineStr"/>
-      <c r="E10" s="22" t="inlineStr">
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>🟠 중요</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
+        <is>
+          <t>가격 구조 미확정</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>별첨 III 완성 전 서명 금지 원칙 + 세무 확인</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr"/>
+      <c r="F10" s="28" t="inlineStr">
         <is>
           <t>별첨 완성 시</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1">
-      <c r="A11" s="15" t="n">
+    <row r="11" ht="28" customHeight="1">
+      <c r="A11" s="17" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="19" t="inlineStr">
-        <is>
-          <t>최소 계약 기간</t>
-        </is>
-      </c>
-      <c r="C11" s="20" t="inlineStr">
-        <is>
-          <t>24개월 이상 최소 기간 + 해지 통지 180일 협상 방향 승인</t>
-        </is>
-      </c>
-      <c r="D11" s="21" t="inlineStr"/>
-      <c r="E11" s="22" t="inlineStr">
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>🟠 중요</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>계약 기간 12개월</t>
+        </is>
+      </c>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>최소 24개월 + 해지 통지 180일 협상 방향</t>
+        </is>
+      </c>
+      <c r="E11" s="27" t="inlineStr"/>
+      <c r="F11" s="28" t="inlineStr">
         <is>
           <t>서명 전</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="15" t="n">
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="17" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>별첨 I(BOM·제품사양) 완성</t>
-        </is>
-      </c>
-      <c r="C12" s="20" t="inlineStr">
-        <is>
-          <t>별첨 I 완성 전 서명 절대 금지 원칙 수립 + BOM 수령 일정 확인</t>
-        </is>
-      </c>
-      <c r="D12" s="21" t="inlineStr"/>
-      <c r="E12" s="22" t="inlineStr">
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>🟠 중요</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>Appendix I 공란</t>
+        </is>
+      </c>
+      <c r="D12" s="26" t="inlineStr">
+        <is>
+          <t>별첨 I 완성 전 서명 금지 원칙 확립</t>
+        </is>
+      </c>
+      <c r="E12" s="27" t="inlineStr"/>
+      <c r="F12" s="28" t="inlineStr">
         <is>
           <t>별첨 완성 시</t>
         </is>
@@ -1503,7 +1693,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>